<commit_message>
Invoice UI Refresh: R417 foreign-vs-ours reconciliation + resolve PO-1 (v45)
Read-only Rule 38/39 reconciliation of the 30 foreign (creator-6) cases in
R417: all complementary, 0 contradictions; nothing edited on either side.
PO-1 resolved by spec v45 (Terminology rewritten to the open-balance
definition = S11-R6a); PO sheet annotated on both tabs; PROJECT-STATE updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QvLHRX1rY5c7HuyoMWVGpU
</commit_message>
<xml_diff>
--- a/build/invoice-ui-refresh/questions-2026-08-25/Questions-for-Chris-Ward_Invoice-UI-Refresh_2026-08-25.xlsx
+++ b/build/invoice-ui-refresh/questions-2026-08-25/Questions-for-Chris-Ward_Invoice-UI-Refresh_2026-08-25.xlsx
@@ -463,6 +463,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -521,7 +522,11 @@
           <t>A) Show the remaining credit (positive), $0.00 only when used up or voided - and we will correct the glossary line.   B) Show what the glossary says - and we will rewrite the affected test cases.</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>RESOLVED BY SPEC v45 (Confluence 755990532, change-log entry 2026-08-27): the Terminology "Balance" for the Credit Invoice was rewritten to the open-balance definition, matching S11-R6a and Option A. The v39 conflict that prompted this question no longer exists, so no answer is needed. Our case INV-CRED-06 (C44969) already reflects this. — QA, 2026-08-31</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="120" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -579,6 +584,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -624,7 +630,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Authored to S11-R6a (open balance); Rule 32 latest/specific wins; glossary line stale</t>
+          <t>Authored to S11-R6a (open balance); Rule 32 latest/specific wins; glossary line stale | STATUS 2026-08-31: RESOLVED by spec v45 (Terminology rewritten to open-balance = S11-R6a, change-log 2026-08-27). Question moot; do not send.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">

</xml_diff>